<commit_message>
v0.2 added FASTLED compatible leds
</commit_message>
<xml_diff>
--- a/hardware/boards/brain/BOM_brain.xlsx
+++ b/hardware/boards/brain/BOM_brain.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_LCSC ESP32S3R8N8 Dev Board " state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_ESP32S3R8N8 brain_brain_202" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="319">
   <si>
     <t>No.</t>
   </si>
@@ -523,7 +523,7 @@
     <t>220Ω</t>
   </si>
   <si>
-    <t>R1,R4,R5,R6,R7,R32</t>
+    <t>R1,R4,R5,R6,R7,R8,R32</t>
   </si>
   <si>
     <t>0402WGF2200TCE</t>
@@ -784,6 +784,27 @@
     <t>37</t>
   </si>
   <si>
+    <t>SN74AHCT1G125DBVR(UMW)</t>
+  </si>
+  <si>
+    <t>U6</t>
+  </si>
+  <si>
+    <t>SOT-23-5_L3.0-W1.5-P0.95-LS2.8-BL</t>
+  </si>
+  <si>
+    <t>UMW(友台半导体)</t>
+  </si>
+  <si>
+    <t>C20617903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logic Type:- Number of Gates:1 Voltage - Supply:4.5V~5.5V Voltage - Supply:4.5V~5.5V Quiescent Current:10uA Current - Output Low(IOL):8mA Current - Output High(IOH):8mA Input Logic Level - High:2V Input Logic Level - High:2V Input Logic Level - Low:800mV </t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
     <t>MCP2562-E/SN</t>
   </si>
   <si>
@@ -802,7 +823,7 @@
     <t>Type:Transceiver Supply Voltage:4.5V~5.5V Supply Voltage:4.5V~5.5V</t>
   </si>
   <si>
-    <t>38</t>
+    <t>39</t>
   </si>
   <si>
     <t>PCA9306DCUR</t>
@@ -820,7 +841,7 @@
     <t>Channel Type:Bi-Directional Number of Channels:2 Supply Voltage (VCCA):1.2V~3.3V Supply Voltage (VCCA):1.2V~3.3V Supply Voltage (VCCB):1.8V~5.5V Supply Voltage (VCCB):1.8V~5.5V Input Signal:- Output Signal:- Output Type:Open Drain，Push-pull Data Rate:- Op</t>
   </si>
   <si>
-    <t>39</t>
+    <t>40</t>
   </si>
   <si>
     <t>RFANT5220110A0T</t>
@@ -841,7 +862,7 @@
     <t>2.4 GHz 陶瓷天线</t>
   </si>
   <si>
-    <t>40</t>
+    <t>41</t>
   </si>
   <si>
     <t>NCV68061SNAIT1G</t>
@@ -859,7 +880,7 @@
     <t>C5206748</t>
   </si>
   <si>
-    <t>41</t>
+    <t>42</t>
   </si>
   <si>
     <t>TPS5430DDAR</t>
@@ -877,7 +898,7 @@
     <t>Function:Buck Voltage - Supply:5.5V~36V Voltage - Supply:5.5V~36V Output Voltage:1.221V~32.04V Output Voltage:1.221V~32.04V Output Current:3A Frequency - Switching:500kHz Frequency - Switching:500kHz Operating Temperature:-40℃~+125℃@(TJ) Operating Tempera</t>
   </si>
   <si>
-    <t>42</t>
+    <t>43</t>
   </si>
   <si>
     <t>EL3H7(B)(TA)-G</t>
@@ -901,7 +922,7 @@
     <t>Input type:DC Output Type:Phototransistor Voltage - Forward(Vf):1.2V Output Current:50mA Isolation Voltage(Vrms):3.75kV Reverse Voltage:6V Load Voltage:80V Vce Saturation(VCE(sat)):200mV@10mA,1mA Rise time:5us Fall time:3us Operating Temperature:-55℃~+110</t>
   </si>
   <si>
-    <t>43</t>
+    <t>44</t>
   </si>
   <si>
     <t>AMS1117-3.3</t>
@@ -925,7 +946,7 @@
     <t>Output Type:Fixed Voltage - Supply:16V Output Voltage:3.3V Output Voltage:3.3V Output Current:1A Power Supply Rejection Ratio (PSRR):72dB@(120Hz) Voltage Dropout:1.1V@(800mA) standby current:5mA Noise:0.003%Vout Features:Over Current Protection；Over Tempe</t>
   </si>
   <si>
-    <t>44</t>
+    <t>45</t>
   </si>
   <si>
     <t>40MHz</t>
@@ -1323,7 +1344,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="15" width="20" customWidth="1"/>
@@ -2415,7 +2436,7 @@
         <v>168</v>
       </c>
       <c r="B24">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C24" t="s">
         <v>169</v>
@@ -3138,10 +3159,10 @@
         <v>264</v>
       </c>
       <c r="H39" t="s">
-        <v>228</v>
+        <v>267</v>
       </c>
       <c r="I39" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="J39" t="s">
         <v>22</v>
@@ -3153,7 +3174,7 @@
         <v>264</v>
       </c>
       <c r="M39" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="N39" t="s">
         <v>24</v>
@@ -3164,28 +3185,28 @@
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B40">
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D40" t="s">
+        <v>272</v>
+      </c>
+      <c r="E40" t="s">
+        <v>273</v>
+      </c>
+      <c r="F40" t="s">
+        <v>24</v>
+      </c>
+      <c r="G40" t="s">
         <v>271</v>
       </c>
-      <c r="E40" t="s">
-        <v>272</v>
-      </c>
-      <c r="F40" t="s">
-        <v>24</v>
-      </c>
-      <c r="G40" t="s">
-        <v>270</v>
-      </c>
       <c r="H40" t="s">
-        <v>273</v>
+        <v>228</v>
       </c>
       <c r="I40" t="s">
         <v>274</v>
@@ -3194,10 +3215,10 @@
         <v>22</v>
       </c>
       <c r="K40" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L40" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="M40" t="s">
         <v>275</v>
@@ -3247,7 +3268,7 @@
         <v>277</v>
       </c>
       <c r="M41" t="s">
-        <v>24</v>
+        <v>282</v>
       </c>
       <c r="N41" t="s">
         <v>24</v>
@@ -3258,43 +3279,43 @@
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B42">
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D42" t="s">
+        <v>285</v>
+      </c>
+      <c r="E42" t="s">
+        <v>286</v>
+      </c>
+      <c r="F42" t="s">
+        <v>24</v>
+      </c>
+      <c r="G42" t="s">
         <v>284</v>
       </c>
-      <c r="E42" t="s">
-        <v>285</v>
-      </c>
-      <c r="F42" t="s">
-        <v>24</v>
-      </c>
-      <c r="G42" t="s">
-        <v>283</v>
-      </c>
       <c r="H42" t="s">
-        <v>228</v>
+        <v>287</v>
       </c>
       <c r="I42" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="J42" t="s">
         <v>22</v>
       </c>
       <c r="K42" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="L42" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="M42" t="s">
-        <v>287</v>
+        <v>24</v>
       </c>
       <c r="N42" t="s">
         <v>24</v>
@@ -3305,28 +3326,28 @@
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B43">
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D43" t="s">
+        <v>291</v>
+      </c>
+      <c r="E43" t="s">
+        <v>292</v>
+      </c>
+      <c r="F43" t="s">
+        <v>24</v>
+      </c>
+      <c r="G43" t="s">
         <v>290</v>
       </c>
-      <c r="E43" t="s">
-        <v>291</v>
-      </c>
-      <c r="F43" t="s">
-        <v>24</v>
-      </c>
-      <c r="G43" t="s">
-        <v>289</v>
-      </c>
       <c r="H43" t="s">
-        <v>292</v>
+        <v>228</v>
       </c>
       <c r="I43" t="s">
         <v>293</v>
@@ -3335,13 +3356,13 @@
         <v>22</v>
       </c>
       <c r="K43" t="s">
+        <v>290</v>
+      </c>
+      <c r="L43" t="s">
+        <v>290</v>
+      </c>
+      <c r="M43" t="s">
         <v>294</v>
-      </c>
-      <c r="L43" t="s">
-        <v>289</v>
-      </c>
-      <c r="M43" t="s">
-        <v>295</v>
       </c>
       <c r="N43" t="s">
         <v>24</v>
@@ -3352,43 +3373,43 @@
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B44">
         <v>1</v>
       </c>
       <c r="C44" t="s">
+        <v>296</v>
+      </c>
+      <c r="D44" t="s">
         <v>297</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>298</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
+        <v>24</v>
+      </c>
+      <c r="G44" t="s">
+        <v>296</v>
+      </c>
+      <c r="H44" t="s">
         <v>299</v>
       </c>
-      <c r="F44" t="s">
-        <v>24</v>
-      </c>
-      <c r="G44" t="s">
-        <v>297</v>
-      </c>
-      <c r="H44" t="s">
+      <c r="I44" t="s">
         <v>300</v>
       </c>
-      <c r="I44" t="s">
+      <c r="J44" t="s">
+        <v>22</v>
+      </c>
+      <c r="K44" t="s">
         <v>301</v>
       </c>
-      <c r="J44" t="s">
-        <v>22</v>
-      </c>
-      <c r="K44" t="s">
+      <c r="L44" t="s">
+        <v>296</v>
+      </c>
+      <c r="M44" t="s">
         <v>302</v>
-      </c>
-      <c r="L44" t="s">
-        <v>297</v>
-      </c>
-      <c r="M44" t="s">
-        <v>303</v>
       </c>
       <c r="N44" t="s">
         <v>24</v>
@@ -3399,53 +3420,100 @@
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B45">
         <v>1</v>
       </c>
       <c r="C45" t="s">
+        <v>304</v>
+      </c>
+      <c r="D45" t="s">
         <v>305</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>306</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
+        <v>24</v>
+      </c>
+      <c r="G45" t="s">
+        <v>304</v>
+      </c>
+      <c r="H45" t="s">
         <v>307</v>
       </c>
-      <c r="F45" t="s">
-        <v>305</v>
-      </c>
-      <c r="G45" t="s">
+      <c r="I45" t="s">
         <v>308</v>
       </c>
-      <c r="H45" t="s">
+      <c r="J45" t="s">
+        <v>22</v>
+      </c>
+      <c r="K45" t="s">
         <v>309</v>
       </c>
-      <c r="I45" t="s">
+      <c r="L45" t="s">
+        <v>304</v>
+      </c>
+      <c r="M45" t="s">
         <v>310</v>
       </c>
-      <c r="J45" t="s">
-        <v>22</v>
-      </c>
-      <c r="K45" t="s">
-        <v>308</v>
-      </c>
-      <c r="L45" t="s">
-        <v>305</v>
-      </c>
-      <c r="M45" t="s">
+      <c r="N45" t="s">
+        <v>24</v>
+      </c>
+      <c r="O45" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>311</v>
       </c>
-      <c r="N45" t="s">
-        <v>24</v>
-      </c>
-      <c r="O45" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>312</v>
+      </c>
+      <c r="D46" t="s">
+        <v>313</v>
+      </c>
+      <c r="E46" t="s">
+        <v>314</v>
+      </c>
+      <c r="F46" t="s">
+        <v>312</v>
+      </c>
+      <c r="G46" t="s">
+        <v>315</v>
+      </c>
+      <c r="H46" t="s">
+        <v>316</v>
+      </c>
+      <c r="I46" t="s">
+        <v>317</v>
+      </c>
+      <c r="J46" t="s">
+        <v>22</v>
+      </c>
+      <c r="K46" t="s">
+        <v>315</v>
+      </c>
+      <c r="L46" t="s">
+        <v>312</v>
+      </c>
+      <c r="M46" t="s">
+        <v>318</v>
+      </c>
+      <c r="N46" t="s">
+        <v>24</v>
+      </c>
+      <c r="O46" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Substitute out-of-stock parts on brain and handgrip boards
Brain: replace NCV68061 ideal diode controller with LM74700-Q1 (U7) and
add C3. Handgrip: replace SK6805-EC15 LEDs with SK6805D-EC2018.
Updated Gerbers, BOMs, pick-and-place files and brain PCB PDF.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/boards/brain/BOM_brain.xlsx
+++ b/hardware/boards/brain/BOM_brain.xlsx
@@ -112,6 +112,27 @@
     <t>3</t>
   </si>
   <si>
+    <t>C3,C51,C52,C55,C58</t>
+  </si>
+  <si>
+    <t>C0603</t>
+  </si>
+  <si>
+    <t>CC0603KRX7R9BB104</t>
+  </si>
+  <si>
+    <t>YAGEO(国巨)</t>
+  </si>
+  <si>
+    <t>C14663</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacitance:100nF Tolerance:±10% Tolerance:±10% Voltage Rating:50V Temperature Coefficient:X7R </t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
     <t>C19,C20,C21,C22,C23</t>
   </si>
   <si>
@@ -130,7 +151,7 @@
     <t>容值:100nF;精度:±10%;额定电压:50V;材质(温度系数):X7R;</t>
   </si>
   <si>
-    <t>4</t>
+    <t>5</t>
   </si>
   <si>
     <t>1uF</t>
@@ -148,7 +169,7 @@
     <t>容值:1uF;精度:±10%;额定电压:10V;材质(温度系数):X5R;</t>
   </si>
   <si>
-    <t>5</t>
+    <t>6</t>
   </si>
   <si>
     <t>10pF</t>
@@ -166,7 +187,7 @@
     <t>容值:10pF;精度:±5%;额定电压:50V;材质(温度系数):C0G;</t>
   </si>
   <si>
-    <t>6</t>
+    <t>7</t>
   </si>
   <si>
     <t>10uF</t>
@@ -184,7 +205,7 @@
     <t xml:space="preserve">Capacitance:10uF Tolerance:±10% Tolerance:±10% Voltage Rating:50V Temperature Coefficient:X5R </t>
   </si>
   <si>
-    <t>7</t>
+    <t>8</t>
   </si>
   <si>
     <t>10nF</t>
@@ -202,27 +223,6 @@
     <t>C76702</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>C51,C52,C55,C58</t>
-  </si>
-  <si>
-    <t>C0603</t>
-  </si>
-  <si>
-    <t>CC0603KRX7R9BB104</t>
-  </si>
-  <si>
-    <t>YAGEO(国巨)</t>
-  </si>
-  <si>
-    <t>C14663</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capacitance:100nF Tolerance:±10% Tolerance:±10% Voltage Rating:50V Temperature Coefficient:X7R </t>
-  </si>
-  <si>
     <t>9</t>
   </si>
   <si>
@@ -805,6 +805,24 @@
     <t>38</t>
   </si>
   <si>
+    <t>LM74700QDBVRQ1</t>
+  </si>
+  <si>
+    <t>U7</t>
+  </si>
+  <si>
+    <t>SOT-23-6_L2.9-W1.6-P0.95-LS2.8-BL</t>
+  </si>
+  <si>
+    <t>C2941042</t>
+  </si>
+  <si>
+    <t>LM74700QDBVRQ1_C2941042</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
     <t>MCP2562-E/SN</t>
   </si>
   <si>
@@ -823,7 +841,7 @@
     <t>Type:Transceiver Supply Voltage:4.5V~5.5V Supply Voltage:4.5V~5.5V</t>
   </si>
   <si>
-    <t>39</t>
+    <t>40</t>
   </si>
   <si>
     <t>PCA9306DCUR</t>
@@ -841,7 +859,7 @@
     <t>Channel Type:Bi-Directional Number of Channels:2 Supply Voltage (VCCA):1.2V~3.3V Supply Voltage (VCCA):1.2V~3.3V Supply Voltage (VCCB):1.8V~5.5V Supply Voltage (VCCB):1.8V~5.5V Input Signal:- Output Signal:- Output Type:Open Drain，Push-pull Data Rate:- Op</t>
   </si>
   <si>
-    <t>40</t>
+    <t>41</t>
   </si>
   <si>
     <t>RFANT5220110A0T</t>
@@ -860,24 +878,6 @@
   </si>
   <si>
     <t>2.4 GHz 陶瓷天线</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
-    <t>NCV68061SNAIT1G</t>
-  </si>
-  <si>
-    <t>U26</t>
-  </si>
-  <si>
-    <t>TSOP-6_L3.0-W1.5-P0.95-BL</t>
-  </si>
-  <si>
-    <t>onsemi(安森美)</t>
-  </si>
-  <si>
-    <t>C5206748</t>
   </si>
   <si>
     <t>42</t>
@@ -1543,28 +1543,28 @@
         <v>39</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
         <v>40</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>41</v>
       </c>
-      <c r="E5" t="s">
-        <v>34</v>
-      </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="G5" t="s">
         <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="I5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J5" t="s">
         <v>22</v>
@@ -1573,10 +1573,10 @@
         <v>42</v>
       </c>
       <c r="L5" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="M5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N5" t="s">
         <v>24</v>
@@ -1587,43 +1587,43 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" t="s">
         <v>47</v>
       </c>
-      <c r="E6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" t="s">
-        <v>46</v>
-      </c>
       <c r="G6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H6" t="s">
         <v>20</v>
       </c>
       <c r="I6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" t="s">
         <v>49</v>
       </c>
-      <c r="J6" t="s">
-        <v>22</v>
-      </c>
-      <c r="K6" t="s">
-        <v>48</v>
-      </c>
       <c r="L6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N6" t="s">
         <v>24</v>
@@ -1634,43 +1634,43 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" t="s">
         <v>53</v>
       </c>
-      <c r="E7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" t="s">
-        <v>52</v>
-      </c>
       <c r="G7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H7" t="s">
         <v>20</v>
       </c>
       <c r="I7" t="s">
+        <v>56</v>
+      </c>
+      <c r="J7" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" t="s">
         <v>55</v>
       </c>
-      <c r="J7" t="s">
-        <v>22</v>
-      </c>
-      <c r="K7" t="s">
-        <v>54</v>
-      </c>
       <c r="L7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N7" t="s">
         <v>24</v>
@@ -1681,28 +1681,28 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" t="s">
         <v>59</v>
       </c>
-      <c r="E8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" t="s">
-        <v>58</v>
-      </c>
       <c r="G8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="I8" t="s">
         <v>62</v>
@@ -1711,13 +1711,13 @@
         <v>22</v>
       </c>
       <c r="K8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M8" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="N8" t="s">
         <v>24</v>
@@ -1728,43 +1728,43 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="D9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" t="s">
         <v>65</v>
       </c>
-      <c r="F9" t="s">
-        <v>16</v>
-      </c>
       <c r="G9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H9" t="s">
+        <v>68</v>
+      </c>
+      <c r="I9" t="s">
+        <v>69</v>
+      </c>
+      <c r="J9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9" t="s">
         <v>67</v>
       </c>
-      <c r="I9" t="s">
-        <v>68</v>
-      </c>
-      <c r="J9" t="s">
-        <v>22</v>
-      </c>
-      <c r="K9" t="s">
-        <v>66</v>
-      </c>
       <c r="L9" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="M9" t="s">
-        <v>69</v>
+        <v>23</v>
       </c>
       <c r="N9" t="s">
         <v>24</v>
@@ -2116,7 +2116,7 @@
         <v>122</v>
       </c>
       <c r="E17" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F17" t="s">
         <v>121</v>
@@ -2125,7 +2125,7 @@
         <v>123</v>
       </c>
       <c r="H17" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="I17" t="s">
         <v>124</v>
@@ -2445,7 +2445,7 @@
         <v>170</v>
       </c>
       <c r="E24" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F24" t="s">
         <v>169</v>
@@ -2539,7 +2539,7 @@
         <v>184</v>
       </c>
       <c r="E26" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F26" t="s">
         <v>183</v>
@@ -2586,7 +2586,7 @@
         <v>190</v>
       </c>
       <c r="E27" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F27" t="s">
         <v>189</v>
@@ -2633,7 +2633,7 @@
         <v>196</v>
       </c>
       <c r="E28" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F28" t="s">
         <v>195</v>
@@ -2680,7 +2680,7 @@
         <v>202</v>
       </c>
       <c r="E29" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F29" t="s">
         <v>201</v>
@@ -2727,7 +2727,7 @@
         <v>207</v>
       </c>
       <c r="E30" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F30" t="s">
         <v>176</v>
@@ -3159,22 +3159,22 @@
         <v>264</v>
       </c>
       <c r="H39" t="s">
+        <v>228</v>
+      </c>
+      <c r="I39" t="s">
         <v>267</v>
       </c>
-      <c r="I39" t="s">
+      <c r="J39" t="s">
+        <v>22</v>
+      </c>
+      <c r="K39" t="s">
         <v>268</v>
-      </c>
-      <c r="J39" t="s">
-        <v>22</v>
-      </c>
-      <c r="K39" t="s">
-        <v>264</v>
       </c>
       <c r="L39" t="s">
         <v>264</v>
       </c>
       <c r="M39" t="s">
-        <v>269</v>
+        <v>24</v>
       </c>
       <c r="N39" t="s">
         <v>24</v>
@@ -3185,28 +3185,28 @@
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B40">
         <v>1</v>
       </c>
       <c r="C40" t="s">
+        <v>270</v>
+      </c>
+      <c r="D40" t="s">
         <v>271</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>272</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
+        <v>24</v>
+      </c>
+      <c r="G40" t="s">
+        <v>270</v>
+      </c>
+      <c r="H40" t="s">
         <v>273</v>
-      </c>
-      <c r="F40" t="s">
-        <v>24</v>
-      </c>
-      <c r="G40" t="s">
-        <v>271</v>
-      </c>
-      <c r="H40" t="s">
-        <v>228</v>
       </c>
       <c r="I40" t="s">
         <v>274</v>
@@ -3215,10 +3215,10 @@
         <v>22</v>
       </c>
       <c r="K40" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="L40" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="M40" t="s">
         <v>275</v>
@@ -3253,10 +3253,10 @@
         <v>277</v>
       </c>
       <c r="H41" t="s">
+        <v>228</v>
+      </c>
+      <c r="I41" t="s">
         <v>280</v>
-      </c>
-      <c r="I41" t="s">
-        <v>281</v>
       </c>
       <c r="J41" t="s">
         <v>22</v>
@@ -3268,7 +3268,7 @@
         <v>277</v>
       </c>
       <c r="M41" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="N41" t="s">
         <v>24</v>
@@ -3279,43 +3279,43 @@
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B42">
         <v>1</v>
       </c>
       <c r="C42" t="s">
+        <v>283</v>
+      </c>
+      <c r="D42" t="s">
         <v>284</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>285</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
+        <v>24</v>
+      </c>
+      <c r="G42" t="s">
+        <v>283</v>
+      </c>
+      <c r="H42" t="s">
         <v>286</v>
       </c>
-      <c r="F42" t="s">
-        <v>24</v>
-      </c>
-      <c r="G42" t="s">
-        <v>284</v>
-      </c>
-      <c r="H42" t="s">
+      <c r="I42" t="s">
         <v>287</v>
       </c>
-      <c r="I42" t="s">
+      <c r="J42" t="s">
+        <v>22</v>
+      </c>
+      <c r="K42" t="s">
+        <v>283</v>
+      </c>
+      <c r="L42" t="s">
+        <v>283</v>
+      </c>
+      <c r="M42" t="s">
         <v>288</v>
-      </c>
-      <c r="J42" t="s">
-        <v>22</v>
-      </c>
-      <c r="K42" t="s">
-        <v>284</v>
-      </c>
-      <c r="L42" t="s">
-        <v>284</v>
-      </c>
-      <c r="M42" t="s">
-        <v>24</v>
       </c>
       <c r="N42" t="s">
         <v>24</v>

</xml_diff>